<commit_message>
Agentic GraphRAG integree avec succes
</commit_message>
<xml_diff>
--- a/data/raw/demandeur.xlsx
+++ b/data/raw/demandeur.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA SCIENCES\PRE-TEST-SYSTEME-DE-RECOMMANDATION\data\emploi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA SCIENCES\SYSTEME-DE-RECOMMANDATION-HYBRIDE-\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF12C570-801C-43FF-A118-6539513389BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F6A26F9-E2CD-4EE0-9210-031F5C487062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8E6E5ED4-7FCF-4E43-BD2F-629EB294BB13}"/>
   </bookViews>
@@ -6716,6 +6716,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.1796875" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
     <col min="14" max="14" width="14.54296875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>